<commit_message>
Pass foo and foo_units
</commit_message>
<xml_diff>
--- a/tests/conformance_tests/foo_units/test_scripts/TestScript-foo-units.xlsx
+++ b/tests/conformance_tests/foo_units/test_scripts/TestScript-foo-units.xlsx
@@ -3872,7 +3872,7 @@
         <v>74</v>
       </c>
       <c r="C34" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D34" s="40" t="s">
         <v>80</v>
@@ -3974,7 +3974,7 @@
         <v>81</v>
       </c>
       <c r="C35" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D35" s="40" t="s">
         <v>80</v>
@@ -4076,7 +4076,7 @@
         <v>82</v>
       </c>
       <c r="C36" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D36" s="40" t="s">
         <v>80</v>
@@ -4178,7 +4178,7 @@
         <v>83</v>
       </c>
       <c r="C37" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D37" s="40" t="s">
         <v>80</v>
@@ -4280,7 +4280,7 @@
         <v>84</v>
       </c>
       <c r="C38" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D38" s="40" t="s">
         <v>80</v>
@@ -4994,7 +4994,7 @@
         <v>91</v>
       </c>
       <c r="C45" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D45" s="40" t="s">
         <v>80</v>
@@ -5029,7 +5029,7 @@
         <v>92</v>
       </c>
       <c r="C46" s="53" t="n">
-        <v>1E-006</v>
+        <v>0.0001</v>
       </c>
       <c r="D46" s="40" t="s">
         <v>80</v>
@@ -5059,7 +5059,7 @@
   </sheetData>
   <conditionalFormatting sqref="M34:ZY44 L8:ZY27 G28:ZY28 L34:L38 L41:L44">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>#ref!&lt;&gt;#REF!</formula>
+      <formula>#ref!&lt;&gt;#ref!</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>